<commit_message>
Avances 23/04: estimación de 50 iteraciones
</commit_message>
<xml_diff>
--- a/Códigos_oficiales/codigos_optimizacion/hiperparametros/resultados_cv_pso_20260410_125509/cv_fold_results - copia 2.xlsx
+++ b/Códigos_oficiales/codigos_optimizacion/hiperparametros/resultados_cv_pso_20260410_125509/cv_fold_results - copia 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-mfolch\Documents\Proyecto_Tintos_CyT\Códigos_oficiales\codigos_optimizacion\hiperparametros\resultados_cv_pso_20260410_125509\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3D8AD4A-0C87-4F23-BE73-C39EE8A7E552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA992039-271E-4729-867F-D13E7B27833F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$O$1</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">Hoja1!$B$12:$B$16</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Hoja1!$B$17:$B$21</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Hoja1!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Hoja1!$D$17:$D$21</definedName>
     <definedName name="_xlchart.v1.10" hidden="1">Hoja1!$F$2</definedName>
     <definedName name="_xlchart.v1.11" hidden="1">Hoja1!$F$3</definedName>
     <definedName name="_xlchart.v1.12" hidden="1">Hoja1!$F$4</definedName>
@@ -28,31 +28,70 @@
     <definedName name="_xlchart.v1.15" hidden="1">Hoja1!$F$7</definedName>
     <definedName name="_xlchart.v1.16" hidden="1">Hoja1!$F$8</definedName>
     <definedName name="_xlchart.v1.17" hidden="1">Hoja1!$F$9</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">Hoja1!$D$12:$D$16</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">Hoja1!$D$17:$D$21</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Hoja1!$B$22:$B$26</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">Hoja1!$D$22:$D$26</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">Hoja1!$D$27:$D$31</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">Hoja1!$D$2:$D$6</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">Hoja1!$D$32:$D$36</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">Hoja1!$D$37:$D$41</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">Hoja1!$D$42:$D$46</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">Hoja1!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">Hoja1!$B$12:$B$16</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">Hoja1!$B$17:$B$21</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Hoja1!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">Hoja1!$B$22:$B$26</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">Hoja1!$B$27:$B$31</definedName>
+    <definedName name="_xlchart.v1.22" hidden="1">Hoja1!$B$2:$B$6</definedName>
+    <definedName name="_xlchart.v1.23" hidden="1">Hoja1!$B$32:$B$36</definedName>
+    <definedName name="_xlchart.v1.24" hidden="1">Hoja1!$B$37:$B$41</definedName>
+    <definedName name="_xlchart.v1.25" hidden="1">Hoja1!$B$42:$B$46</definedName>
+    <definedName name="_xlchart.v1.26" hidden="1">Hoja1!$B$7:$B$11</definedName>
     <definedName name="_xlchart.v1.27" hidden="1">Hoja1!$F$10</definedName>
     <definedName name="_xlchart.v1.28" hidden="1">Hoja1!$F$2</definedName>
     <definedName name="_xlchart.v1.29" hidden="1">Hoja1!$F$3</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Hoja1!$B$27:$B$31</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Hoja1!$D$27:$D$31</definedName>
     <definedName name="_xlchart.v1.30" hidden="1">Hoja1!$F$4</definedName>
     <definedName name="_xlchart.v1.31" hidden="1">Hoja1!$F$5</definedName>
     <definedName name="_xlchart.v1.32" hidden="1">Hoja1!$F$6</definedName>
     <definedName name="_xlchart.v1.33" hidden="1">Hoja1!$F$7</definedName>
     <definedName name="_xlchart.v1.34" hidden="1">Hoja1!$F$8</definedName>
     <definedName name="_xlchart.v1.35" hidden="1">Hoja1!$F$9</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Hoja1!$B$2:$B$6</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Hoja1!$B$32:$B$36</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Hoja1!$B$37:$B$41</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Hoja1!$B$42:$B$46</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Hoja1!$B$7:$B$11</definedName>
+    <definedName name="_xlchart.v1.36" hidden="1">Hoja1!$M$19</definedName>
+    <definedName name="_xlchart.v1.37" hidden="1">Hoja1!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.38" hidden="1">Hoja1!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.39" hidden="1">Hoja1!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Hoja1!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.40" hidden="1">Hoja1!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.41" hidden="1">Hoja1!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.42" hidden="1">Hoja1!$C$32:$C$36</definedName>
+    <definedName name="_xlchart.v1.43" hidden="1">Hoja1!$C$37:$C$41</definedName>
+    <definedName name="_xlchart.v1.44" hidden="1">Hoja1!$C$42:$C$46</definedName>
+    <definedName name="_xlchart.v1.45" hidden="1">Hoja1!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.46" hidden="1">Hoja1!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.47" hidden="1">Hoja1!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.48" hidden="1">Hoja1!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.49" hidden="1">Hoja1!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Hoja1!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.50" hidden="1">Hoja1!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.51" hidden="1">Hoja1!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.52" hidden="1">Hoja1!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.53" hidden="1">Hoja1!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.54" hidden="1">Hoja1!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.55" hidden="1">Hoja1!$M$19</definedName>
+    <definedName name="_xlchart.v1.56" hidden="1">Hoja1!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.57" hidden="1">Hoja1!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.58" hidden="1">Hoja1!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.59" hidden="1">Hoja1!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Hoja1!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.60" hidden="1">Hoja1!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.61" hidden="1">Hoja1!$C$32:$C$36</definedName>
+    <definedName name="_xlchart.v1.62" hidden="1">Hoja1!$C$37:$C$41</definedName>
+    <definedName name="_xlchart.v1.63" hidden="1">Hoja1!$C$42:$C$46</definedName>
+    <definedName name="_xlchart.v1.64" hidden="1">Hoja1!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.65" hidden="1">Hoja1!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.66" hidden="1">Hoja1!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.67" hidden="1">Hoja1!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.68" hidden="1">Hoja1!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.69" hidden="1">Hoja1!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Hoja1!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.70" hidden="1">Hoja1!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.71" hidden="1">Hoja1!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.72" hidden="1">Hoja1!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.73" hidden="1">Hoja1!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.74" hidden="1">Hoja1!$M$19</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Hoja1!$D$7:$D$11</definedName>
     <definedName name="_xlchart.v1.9" hidden="1">Hoja1!$F$10</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -634,6 +673,211 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
+        <cx:f>_xlchart.v1.22</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.26</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="2">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.18</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="3">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.19</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="4">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.20</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="5">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.21</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="6">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.23</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="7">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.24</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="8">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.25</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Train cost</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>Train cost</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000001-ABD9-44B0-9997-5991F7E3E07A}" formatIdx="1">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.28</cx:f>
+              <cx:v>1</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000002-ABD9-44B0-9997-5991F7E3E07A}" formatIdx="2">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.29</cx:f>
+              <cx:v>2</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000003-ABD9-44B0-9997-5991F7E3E07A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.30</cx:f>
+              <cx:v>3</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="2"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000004-ABD9-44B0-9997-5991F7E3E07A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.31</cx:f>
+              <cx:v>4</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="3"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000005-ABD9-44B0-9997-5991F7E3E07A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.32</cx:f>
+              <cx:v>5</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="4"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000006-ABD9-44B0-9997-5991F7E3E07A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.33</cx:f>
+              <cx:v>6</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="5"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000007-ABD9-44B0-9997-5991F7E3E07A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.34</cx:f>
+              <cx:v>7</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="6"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000008-ABD9-44B0-9997-5991F7E3E07A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.35</cx:f>
+              <cx:v>8</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="7"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000009-ABD9-44B0-9997-5991F7E3E07A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.27</cx:f>
+              <cx:v>9</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="8"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0" hidden="1">
+        <cx:catScaling gapWidth="1"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+        <cx:numFmt formatCode="0,00" sourceLinked="0"/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="b" align="ctr" overlay="0"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
         <cx:f>_xlchart.v1.4</cx:f>
       </cx:numDim>
     </cx:data>
@@ -682,7 +926,7 @@
     <cx:title pos="t" align="ctr" overlay="0">
       <cx:tx>
         <cx:txData>
-          <cx:v>Train cost</cx:v>
+          <cx:v>Validation cost</cx:v>
         </cx:txData>
       </cx:tx>
       <cx:txPr>
@@ -702,7 +946,7 @@
               </a:solidFill>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>Train cost</a:t>
+            <a:t>Validation cost</a:t>
           </a:r>
         </a:p>
       </cx:txPr>
@@ -818,211 +1062,6 @@
           </cx:layoutPr>
         </cx:series>
       </cx:plotAreaRegion>
-      <cx:axis id="0" hidden="1">
-        <cx:catScaling gapWidth="1"/>
-        <cx:tickLabels/>
-      </cx:axis>
-      <cx:axis id="1">
-        <cx:valScaling/>
-        <cx:majorGridlines/>
-        <cx:tickLabels/>
-        <cx:numFmt formatCode="0,00" sourceLinked="0"/>
-      </cx:axis>
-    </cx:plotArea>
-    <cx:legend pos="b" align="ctr" overlay="0"/>
-  </cx:chart>
-</cx:chartSpace>
-</file>
-
-<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
-<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
-  <cx:chartData>
-    <cx:data id="0">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.22</cx:f>
-      </cx:numDim>
-    </cx:data>
-    <cx:data id="1">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.26</cx:f>
-      </cx:numDim>
-    </cx:data>
-    <cx:data id="2">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.18</cx:f>
-      </cx:numDim>
-    </cx:data>
-    <cx:data id="3">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.19</cx:f>
-      </cx:numDim>
-    </cx:data>
-    <cx:data id="4">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.20</cx:f>
-      </cx:numDim>
-    </cx:data>
-    <cx:data id="5">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.21</cx:f>
-      </cx:numDim>
-    </cx:data>
-    <cx:data id="6">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.23</cx:f>
-      </cx:numDim>
-    </cx:data>
-    <cx:data id="7">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.24</cx:f>
-      </cx:numDim>
-    </cx:data>
-    <cx:data id="8">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.25</cx:f>
-      </cx:numDim>
-    </cx:data>
-  </cx:chartData>
-  <cx:chart>
-    <cx:title pos="t" align="ctr" overlay="0">
-      <cx:tx>
-        <cx:txData>
-          <cx:v>Validation cost</cx:v>
-        </cx:txData>
-      </cx:tx>
-      <cx:txPr>
-        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:sysClr>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>Validation cost</a:t>
-          </a:r>
-        </a:p>
-      </cx:txPr>
-    </cx:title>
-    <cx:plotArea>
-      <cx:plotAreaRegion>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000001-ABD9-44B0-9997-5991F7E3E07A}" formatIdx="1">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.28</cx:f>
-              <cx:v>1</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="0"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000002-ABD9-44B0-9997-5991F7E3E07A}" formatIdx="2">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.29</cx:f>
-              <cx:v>2</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="1"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000003-ABD9-44B0-9997-5991F7E3E07A}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.30</cx:f>
-              <cx:v>3</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="2"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000004-ABD9-44B0-9997-5991F7E3E07A}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.31</cx:f>
-              <cx:v>4</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="3"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000005-ABD9-44B0-9997-5991F7E3E07A}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.32</cx:f>
-              <cx:v>5</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="4"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000006-ABD9-44B0-9997-5991F7E3E07A}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.33</cx:f>
-              <cx:v>6</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="5"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000007-ABD9-44B0-9997-5991F7E3E07A}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.34</cx:f>
-              <cx:v>7</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="6"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000008-ABD9-44B0-9997-5991F7E3E07A}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.35</cx:f>
-              <cx:v>8</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="7"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000009-ABD9-44B0-9997-5991F7E3E07A}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f>_xlchart.v1.27</cx:f>
-              <cx:v>9</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:dataId val="8"/>
-          <cx:layoutPr>
-            <cx:statistics quartileMethod="exclusive"/>
-          </cx:layoutPr>
-        </cx:series>
-      </cx:plotAreaRegion>
       <cx:axis id="0">
         <cx:catScaling gapWidth="1"/>
         <cx:tickLabels/>
@@ -1032,6 +1071,320 @@
         <cx:majorGridlines/>
         <cx:tickLabels/>
         <cx:numFmt formatCode="0,000" sourceLinked="0"/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="b" align="ctr" overlay="0"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx3.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.41</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.50</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="2">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.45</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="3">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.54</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="4">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.37</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="5">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.46</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="6">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.38</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="7">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.47</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="8">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.39</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="9">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.48</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="10">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.40</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="11">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.49</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="12">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.42</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="13">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.51</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="14">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.43</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="15">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.52</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="16">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.44</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="17">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.53</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0"/>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{1801D75C-2FD6-4A43-B32D-40831D46013D}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 1</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000001-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 1</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000002-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 2</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="2"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000003-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 2</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="3"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000004-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 3</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="4"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000005-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 3</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="5"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000006-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 4</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="6"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000007-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 4</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="7"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000008-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 5</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="8"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000009-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 5</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="9"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000A-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 6</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="10"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000B-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 6</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="11"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000C-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 7</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="12"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000D-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 7</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="13"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000E-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 8</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="14"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000F-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 8</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="15"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000010-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>train cost 9</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="16"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000011-9E00-45E3-BCDA-FE3A558046F7}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>val cost 9</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="17"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0" hidden="1">
+        <cx:catScaling gapWidth="1"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+        <cx:numFmt formatCode="General" sourceLinked="0"/>
       </cx:axis>
     </cx:plotArea>
     <cx:legend pos="b" align="ctr" overlay="0"/>
@@ -1119,6 +1472,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
   <cs:axisTitle>
@@ -1635,6 +2028,521 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2278,6 +3186,84 @@
             <a:xfrm>
               <a:off x="4511040" y="5349240"/>
               <a:ext cx="5113020" cy="2975610"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-CL" sz="1100"/>
+                <a:t>Este gráfico no está disponible en su versión de Excel.
+Si edita esta forma o guarda el libro en un formato de archivo diferente, el gráfico no se podrá utilizar.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>640773</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>31172</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>360217</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>138544</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="Gráfico 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BEC0A399-04E3-15C0-C300-62644B4C50BD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="9888682" y="2414154"/>
+              <a:ext cx="6037117" cy="3584863"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>

</xml_diff>